<commit_message>
Update Excel files with manual changes
</commit_message>
<xml_diff>
--- a/sheets/real-estate/storage-deal/storage-deal.xlsx
+++ b/sheets/real-estate/storage-deal/storage-deal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\000_drive_drive\600_PROJECTS\modelstack\sheets\real-estate\storage-deal-v1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\000_drive_drive\600_PROJECTS\modelstack\sheets\real-estate\storage-deal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AED1EF2-6EFC-49F8-B3D4-5C656EEA45F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D51394A-AF81-4EBA-85DD-3EB806BB46CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Facility Overview" sheetId="1" r:id="rId1"/>

</xml_diff>